<commit_message>
Relocate xeno-canto files to subdirectory and update frontend labels to differentiate call source
</commit_message>
<xml_diff>
--- a/Location/species_master.xlsx
+++ b/Location/species_master.xlsx
@@ -693,7 +693,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>/audio/Asian Brown Flycatcher.mp3</t>
+          <t>/audio/xeno-canto/Asian Brown Flycatcher.mp3</t>
         </is>
       </c>
     </row>
@@ -750,7 +750,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>/audio/Asian Emerald Dove.mp3</t>
+          <t>/audio/xeno-canto/Asian Emerald Dove.mp3</t>
         </is>
       </c>
     </row>
@@ -909,7 +909,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>/audio/Bank Swallow.mp3</t>
+          <t>/audio/xeno-canto/Bank Swallow.mp3</t>
         </is>
       </c>
     </row>
@@ -1561,7 +1561,7 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>/audio/Brown-breasted Flycatcher.mp3</t>
+          <t>/audio/xeno-canto/Brown-breasted Flycatcher.mp3</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>/audio/Brown-cheeked Fulvetta.wav</t>
+          <t>/audio/xeno-canto/Brown-cheeked Fulvetta.wav</t>
         </is>
       </c>
     </row>
@@ -2258,7 +2258,7 @@
       </c>
       <c r="K34" t="inlineStr">
         <is>
-          <t>/audio/Common Snipe.mp3</t>
+          <t>/audio/xeno-canto/Common Snipe.mp3</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>/audio/Eurasian Coot.mp3</t>
+          <t>/audio/xeno-canto/Eurasian Coot.mp3</t>
         </is>
       </c>
     </row>
@@ -2694,7 +2694,7 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>/audio/Eurasian Curlew.wav</t>
+          <t>/audio/xeno-canto/Eurasian Curlew.wav</t>
         </is>
       </c>
     </row>
@@ -2857,7 +2857,7 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>/audio/Flame-throated Bulbul.mp3</t>
+          <t>/audio/xeno-canto/Flame-throated Bulbul.mp3</t>
         </is>
       </c>
     </row>
@@ -3338,7 +3338,7 @@
       </c>
       <c r="K54" t="inlineStr">
         <is>
-          <t>/audio/Gray-headed Bulbul.mp3</t>
+          <t>/audio/xeno-canto/Gray-headed Bulbul.mp3</t>
         </is>
       </c>
     </row>
@@ -3774,7 +3774,7 @@
       </c>
       <c r="K62" t="inlineStr">
         <is>
-          <t>/audio/Indian Blue Robin.mp3</t>
+          <t>/audio/xeno-canto/Indian Blue Robin.mp3</t>
         </is>
       </c>
     </row>
@@ -4365,7 +4365,7 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>/audio/Jerdon's Bushlark.mp3</t>
+          <t>/audio/xeno-canto/Jerdon's Bushlark.mp3</t>
         </is>
       </c>
     </row>
@@ -6419,7 +6419,7 @@
       </c>
       <c r="K111" t="inlineStr">
         <is>
-          <t>/audio/Sykes's Warbler.mp3</t>
+          <t>/audio/xeno-canto/Sykes's Warbler.mp3</t>
         </is>
       </c>
     </row>
@@ -6472,7 +6472,7 @@
       </c>
       <c r="K112" t="inlineStr">
         <is>
-          <t>/audio/Taiga Flycatcher.mp3</t>
+          <t>/audio/xeno-canto/Taiga Flycatcher.mp3</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="K116" t="inlineStr">
         <is>
-          <t>/audio/Tree Pipit.mp3</t>
+          <t>/audio/xeno-canto/Tree Pipit.mp3</t>
         </is>
       </c>
     </row>
@@ -6798,7 +6798,7 @@
       </c>
       <c r="K118" t="inlineStr">
         <is>
-          <t>/audio/Verditer Flycatcher.mp3</t>
+          <t>/audio/xeno-canto/Verditer Flycatcher.mp3</t>
         </is>
       </c>
     </row>
@@ -7397,7 +7397,7 @@
       </c>
       <c r="K129" t="inlineStr">
         <is>
-          <t>/audio/Zitting Cisticola.mp3</t>
+          <t>/audio/xeno-canto/Zitting Cisticola.mp3</t>
         </is>
       </c>
     </row>

</xml_diff>